<commit_message>
feat: pobut predictor module + analysis scripts and results
- pobut_predictor.py, predict_all_consumers.py, profile_gas_consumption.py: updated core prediction logic
- profiles/: updated op_profiles, profiles.json, summer_op_means, validation_results + new profile CSVs
- 50+ analysis scripts: backtest, regression, clustering, seasonal bias analysis
- analysis results: xlsx/png outputs for all models
- summer_consumption_analysis.py, summer_analysis_results.txt

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/pobut/data/profiles/profiles_summary.xlsx
+++ b/backend/pobut/data/profiles/profiles_summary.xlsx
@@ -703,7 +703,7 @@
         <v>5</v>
       </c>
       <c r="C2" t="n">
-        <v>32.95031864894722</v>
+        <v>23.87</v>
       </c>
     </row>
     <row r="3">
@@ -716,7 +716,7 @@
         <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>20.24022164913171</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="4">
@@ -729,7 +729,7 @@
         <v>7</v>
       </c>
       <c r="C4" t="n">
-        <v>18.06047934630241</v>
+        <v>14.17</v>
       </c>
     </row>
     <row r="5">
@@ -742,7 +742,7 @@
         <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>18.44764192835831</v>
+        <v>14.81</v>
       </c>
     </row>
     <row r="6">
@@ -755,7 +755,7 @@
         <v>9</v>
       </c>
       <c r="C6" t="n">
-        <v>22.69198752629823</v>
+        <v>18.275</v>
       </c>
     </row>
     <row r="7">
@@ -768,7 +768,7 @@
         <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>19.7300386784492</v>
+        <v>11.68678571428571</v>
       </c>
     </row>
     <row r="8">
@@ -781,7 +781,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>10.50631402984815</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -794,7 +794,7 @@
         <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>10.33150718816905</v>
+        <v>7.68</v>
       </c>
     </row>
     <row r="10">
@@ -807,7 +807,7 @@
         <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>10.90144475708113</v>
+        <v>8.74</v>
       </c>
     </row>
     <row r="11">
@@ -820,7 +820,7 @@
         <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>13.23241697102365</v>
+        <v>9.985862068965517</v>
       </c>
     </row>
     <row r="12">
@@ -833,7 +833,7 @@
         <v>5</v>
       </c>
       <c r="C12" t="n">
-        <v>83.75874676501036</v>
+        <v>72.07375</v>
       </c>
     </row>
     <row r="13">
@@ -846,7 +846,7 @@
         <v>6</v>
       </c>
       <c r="C13" t="n">
-        <v>39.09833333333334</v>
+        <v>41.325</v>
       </c>
     </row>
     <row r="14">
@@ -859,7 +859,7 @@
         <v>7</v>
       </c>
       <c r="C14" t="n">
-        <v>33.58285714285714</v>
+        <v>29.42</v>
       </c>
     </row>
     <row r="15">
@@ -872,7 +872,7 @@
         <v>8</v>
       </c>
       <c r="C15" t="n">
-        <v>33.1927950310559</v>
+        <v>29.18</v>
       </c>
     </row>
     <row r="16">
@@ -885,7 +885,7 @@
         <v>9</v>
       </c>
       <c r="C16" t="n">
-        <v>49.10977011494253</v>
+        <v>54.285</v>
       </c>
     </row>
   </sheetData>
@@ -1404,7 +1404,7 @@
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>-0</v>
+        <v>-0.1151</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -1428,7 +1428,7 @@
         <v>19.7</v>
       </c>
       <c r="Q9" t="n">
-        <v>19.73</v>
+        <v>11.61</v>
       </c>
     </row>
     <row r="10">
@@ -1461,7 +1461,7 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>-0</v>
+        <v>-0.08989999999999999</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -1485,7 +1485,7 @@
         <v>10.5</v>
       </c>
       <c r="Q10" t="n">
-        <v>10.51</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -1518,7 +1518,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>-0</v>
+        <v>-0.1242</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -1542,7 +1542,7 @@
         <v>10.4</v>
       </c>
       <c r="Q11" t="n">
-        <v>10.33</v>
+        <v>7.68</v>
       </c>
     </row>
     <row r="12">
@@ -1575,7 +1575,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>-0</v>
+        <v>-0.0796</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -1599,7 +1599,7 @@
         <v>10.9</v>
       </c>
       <c r="Q12" t="n">
-        <v>10.9</v>
+        <v>8.74</v>
       </c>
     </row>
     <row r="13">
@@ -1632,7 +1632,7 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>-0.0001</v>
+        <v>-0.094</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -1656,7 +1656,7 @@
         <v>13.3</v>
       </c>
       <c r="Q13" t="n">
-        <v>13.23</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="14">
@@ -2294,7 +2294,7 @@
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>-0</v>
+        <v>-0.099</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -2318,7 +2318,7 @@
         <v>32.8</v>
       </c>
       <c r="Q25" t="n">
-        <v>32.95</v>
+        <v>23.55</v>
       </c>
     </row>
     <row r="26">
@@ -2351,7 +2351,7 @@
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>-0.0001</v>
+        <v>-0.055</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -2375,7 +2375,7 @@
         <v>20.1</v>
       </c>
       <c r="Q26" t="n">
-        <v>20.24</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="27">
@@ -2408,7 +2408,7 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>-0</v>
+        <v>-0.0673</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -2432,7 +2432,7 @@
         <v>18</v>
       </c>
       <c r="Q27" t="n">
-        <v>18.06</v>
+        <v>14.17</v>
       </c>
     </row>
     <row r="28">
@@ -2465,7 +2465,7 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>-0</v>
+        <v>-0.0623</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -2489,7 +2489,7 @@
         <v>18.4</v>
       </c>
       <c r="Q28" t="n">
-        <v>18.45</v>
+        <v>14.81</v>
       </c>
     </row>
     <row r="29">
@@ -2522,7 +2522,7 @@
         <v>0</v>
       </c>
       <c r="I29" t="n">
-        <v>-0.0001</v>
+        <v>-0.055</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -2546,7 +2546,7 @@
         <v>22.5</v>
       </c>
       <c r="Q29" t="n">
-        <v>22.69</v>
+        <v>18.28</v>
       </c>
     </row>
     <row r="30">
@@ -2838,19 +2838,19 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>125.4</v>
+        <v>175.8</v>
       </c>
       <c r="E2" t="n">
-        <v>22.36</v>
+        <v>40.06</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.6068</v>
+        <v>-4.5873</v>
       </c>
       <c r="G2" t="n">
         <v>37.2</v>
       </c>
       <c r="H2" t="n">
-        <v>55.75</v>
+        <v>74.90000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -2866,19 +2866,19 @@
         <v>60</v>
       </c>
       <c r="D3" t="n">
-        <v>71.7</v>
+        <v>63</v>
       </c>
       <c r="E3" t="n">
-        <v>39.2</v>
+        <v>39.11</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7439</v>
+        <v>0.743</v>
       </c>
       <c r="G3" t="n">
         <v>126.37</v>
       </c>
       <c r="H3" t="n">
-        <v>117.31</v>
+        <v>116.21</v>
       </c>
     </row>
     <row r="4">
@@ -2894,19 +2894,19 @@
         <v>194</v>
       </c>
       <c r="D4" t="n">
-        <v>239.1</v>
+        <v>227.9</v>
       </c>
       <c r="E4" t="n">
-        <v>48.84</v>
+        <v>48.67</v>
       </c>
       <c r="F4" t="n">
-        <v>0.6787</v>
+        <v>0.6783</v>
       </c>
       <c r="G4" t="n">
         <v>144.74</v>
       </c>
       <c r="H4" t="n">
-        <v>138.93</v>
+        <v>137.18</v>
       </c>
     </row>
     <row r="5">

</xml_diff>